<commit_message>
Add example-filled Excel import template
</commit_message>
<xml_diff>
--- a/public/downloads/catalogue-maison-import-template.xlsx
+++ b/public/downloads/catalogue-maison-import-template.xlsx
@@ -97,7 +97,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr defaultRowHeight="20"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -201,19 +201,229 @@
       </c>
     </row>
     <row r="2" spans="1:16" ht="20" customHeight="1">
-      <c r="A2" t="inlineStr" s="2">
-        <is>
-          <t>Commence ici</t>
+      <c r="A2" t="inlineStr" s="3">
+        <is>
+          <t>Oud Noir Intense</t>
         </is>
       </c>
       <c r="B2" t="inlineStr" s="3">
         <is>
-          <t>Laisse vide si inutile</t>
-        </is>
+          <t>oud-noir-intense</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr" s="3">
+        <is>
+          <t>HB Maison</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr" s="3">
+        <is>
+          <t>Parfum</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr" s="3">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr" s="3">
+        <is>
+          <t>Exemple de fiche parfum masculine à remplacer.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr" s="3">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H2" s="3">
+        <v>1</v>
+      </c>
+      <c r="I2" t="inlineStr" s="3">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr" s="3">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr" s="3">
+        <is>
+          <t>100ml</t>
+        </is>
+      </c>
+      <c r="L2" s="3">
+        <v>45000</v>
+      </c>
+      <c r="M2" t="inlineStr" s="3">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N2" s="3">
+        <v>20</v>
+      </c>
+      <c r="O2" t="inlineStr" s="3">
+        <is>
+          <t>HB-ONI-100</t>
+        </is>
+      </c>
+      <c r="P2" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="20" customHeight="1">
+      <c r="A3" t="inlineStr" s="3">
+        <is>
+          <t>Bougie Ambre Doux</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr" s="3">
+        <is>
+          <t>bougie-ambre-doux</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr" s="3">
+        <is>
+          <t>HB Maison</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr" s="3">
+        <is>
+          <t>Bougie</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr" s="3">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr" s="3">
+        <is>
+          <t>Exemple de fiche bougie à personnaliser.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr" s="3">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H3" s="3">
+        <v>2</v>
+      </c>
+      <c r="I3" t="inlineStr" s="3">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr" s="3">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr" s="3">
+        <is>
+          <t>220g</t>
+        </is>
+      </c>
+      <c r="L3" s="3">
+        <v>22000</v>
+      </c>
+      <c r="M3" t="inlineStr" s="3">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N3" s="3">
+        <v>15</v>
+      </c>
+      <c r="O3" t="inlineStr" s="3">
+        <is>
+          <t>HB-BAD-220</t>
+        </is>
+      </c>
+      <c r="P3" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="20" customHeight="1">
+      <c r="A4" t="inlineStr" s="3">
+        <is>
+          <t>Huile Rose Safran</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="3">
+        <is>
+          <t>huile-rose-safran</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="3">
+        <is>
+          <t>HB Maison</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="3">
+        <is>
+          <t>Huile</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="3">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="3">
+        <is>
+          <t>Exemple d’huile parfumée à remplacer.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr" s="3">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H4" s="3">
+        <v>3</v>
+      </c>
+      <c r="I4" t="inlineStr" s="3">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr" s="3">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr" s="3">
+        <is>
+          <t>50ml</t>
+        </is>
+      </c>
+      <c r="L4" s="3">
+        <v>18000</v>
+      </c>
+      <c r="M4" t="inlineStr" s="3">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N4" s="3">
+        <v>30</v>
+      </c>
+      <c r="O4" t="inlineStr" s="3">
+        <is>
+          <t>HB-HRS-50</t>
+        </is>
+      </c>
+      <c r="P4" s="3">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P2"/>
+  <autoFilter ref="A1:P4"/>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E1048576">
       <formula1>"H,F,U"</formula1>
@@ -227,7 +437,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr defaultRowHeight="20"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -243,68 +453,75 @@
     <row r="3" spans="1:1" ht="20" customHeight="1">
       <c r="A3" t="inlineStr" s="0">
         <is>
-          <t>1. Télécharge le modèle CSV ou Excel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ht="20" customHeight="1">
-      <c r="A4" t="inlineStr" s="0">
-        <is>
-          <t>2. Remplis une ligne par variante. Si un produit a plusieurs tailles, répète le nom et change seulement la taille/prix.</t>
+          <t>Les 3 premières lignes sont des exemples. Remplace-les ou ajoute-en d'autres en gardant la même structure.</t>
         </is>
       </c>
     </row>
     <row r="5" spans="1:1" ht="20" customHeight="1">
       <c r="A5" t="inlineStr" s="0">
         <is>
+          <t>1. Télécharge le modèle CSV ou Excel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="20" customHeight="1">
+      <c r="A6" t="inlineStr" s="0">
+        <is>
+          <t>2. Remplis une ligne par variante. Si un produit a plusieurs tailles, répète le nom et change seulement la taille/prix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="20" customHeight="1">
+      <c r="A7" t="inlineStr" s="0">
+        <is>
           <t>3. Réimporte le fichier depuis la page catalogue maison.</t>
         </is>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="20" customHeight="1">
-      <c r="A7" t="inlineStr" s="4">
+    <row r="9" spans="1:1" ht="20" customHeight="1">
+      <c r="A9" t="inlineStr" s="4">
         <is>
           <t>Champs obligatoires</t>
         </is>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="20" customHeight="1">
-      <c r="A8" t="inlineStr" s="0">
+    <row r="10" spans="1:1" ht="20" customHeight="1">
+      <c r="A10" t="inlineStr" s="0">
         <is>
           <t>nom, slug, marque, categorie, genre, description, taille, prix, stock, ordre</t>
         </is>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="20" customHeight="1">
-      <c r="A10" t="inlineStr" s="4">
+    <row r="12" spans="1:1" ht="20" customHeight="1">
+      <c r="A12" t="inlineStr" s="4">
         <is>
           <t>Valeurs autorisées</t>
         </is>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="20" customHeight="1">
-      <c r="A11" t="inlineStr" s="0">
+    <row r="13" spans="1:1" ht="20" customHeight="1">
+      <c r="A13" t="inlineStr" s="0">
         <is>
           <t>genre = H, F, U</t>
         </is>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="20" customHeight="1">
-      <c r="A12" t="inlineStr" s="0">
+    <row r="14" spans="1:1" ht="20" customHeight="1">
+      <c r="A14" t="inlineStr" s="0">
         <is>
           <t>nouveau = oui / non</t>
         </is>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="20" customHeight="1">
-      <c r="A14" t="inlineStr" s="4">
+    <row r="16" spans="1:1" ht="20" customHeight="1">
+      <c r="A16" t="inlineStr" s="4">
         <is>
           <t>Conseil</t>
         </is>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="20" customHeight="1">
-      <c r="A15" t="inlineStr" s="0">
+    <row r="17" spans="1:1" ht="20" customHeight="1">
+      <c r="A17" t="inlineStr" s="0">
         <is>
           <t>Utilise un slug unique. Exemple: oud-noir-intense, rose-safran, huile-d-ambre.</t>
         </is>

</xml_diff>

<commit_message>
Add raw-name autofill for owner catalogue
</commit_message>
<xml_diff>
--- a/public/downloads/catalogue-maison-import-template.xlsx
+++ b/public/downloads/catalogue-maison-import-template.xlsx
@@ -478,6 +478,13 @@
         </is>
       </c>
     </row>
+    <row r="8" spans="1:1" ht="20" customHeight="1">
+      <c r="A8" t="inlineStr" s="0">
+        <is>
+          <t>4. Si tu n'as que des noms, colle la liste brute dans la page catalogue maison: le système remplit les champs par défaut.</t>
+        </is>
+      </c>
+    </row>
     <row r="9" spans="1:1" ht="20" customHeight="1">
       <c r="A9" t="inlineStr" s="4">
         <is>

</xml_diff>